<commit_message>
update(SetupsAI): consolidated website directory & all-channels master - 2026-10-25 10:47:56
</commit_message>
<xml_diff>
--- a/📊 All_Channels_Websites_Master_List.xlsx
+++ b/📊 All_Channels_Websites_Master_List.xlsx
@@ -481,7 +481,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G115"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -4755,7 +4755,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>

</xml_diff>